<commit_message>
Database apparatus & units check 1.0
</commit_message>
<xml_diff>
--- a/database/databases/Standards_Calc_Database_Finalised.xlsx
+++ b/database/databases/Standards_Calc_Database_Finalised.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\JFC-Embodied-Carbon-App\database\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA120171-3527-4967-B8CF-816FA4FBB381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BABC4F-4E5B-42D8-A082-9B6033764322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="392">
   <si>
     <t>system</t>
   </si>
@@ -968,9 +968,6 @@
   </si>
   <si>
     <t>Smoke Exhaust Fans</t>
-  </si>
-  <si>
-    <t>fans</t>
   </si>
   <si>
     <t>Fire Resistant Ductwork</t>
@@ -1241,7 +1238,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1290,6 +1287,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF66FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1303,7 +1306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1316,12 +1319,19 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF66FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -4209,7 +4219,7 @@
         <v>191</v>
       </c>
       <c r="R1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
@@ -4303,14 +4313,14 @@
       <c r="D5" t="s">
         <v>202</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>202</v>
       </c>
       <c r="F5" t="s">
         <v>195</v>
       </c>
-      <c r="I5" t="s">
-        <v>203</v>
+      <c r="I5" s="12" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
@@ -4341,7 +4351,7 @@
         <v>206</v>
       </c>
       <c r="E7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F7" t="s">
         <v>195</v>
@@ -4573,7 +4583,7 @@
         <v>230</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F18" t="s">
         <v>195</v>
@@ -4616,7 +4626,7 @@
         <v>232</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F20" t="s">
         <v>195</v>
@@ -4685,7 +4695,7 @@
         <v>238</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F23" t="s">
         <v>195</v>
@@ -4768,13 +4778,13 @@
         <v>236</v>
       </c>
       <c r="C27" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>350</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>351</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>195</v>
@@ -4801,12 +4811,12 @@
         <v>248</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F28" t="s">
         <v>195</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="12" t="s">
         <v>74</v>
       </c>
       <c r="P28" t="s">
@@ -4827,13 +4837,13 @@
         <v>250</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F29" t="s">
         <v>195</v>
       </c>
-      <c r="I29" t="s">
-        <v>74</v>
+      <c r="I29" s="12" t="s">
+        <v>255</v>
       </c>
       <c r="P29" t="s">
         <v>249</v>
@@ -4853,13 +4863,13 @@
         <v>251</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F30" t="s">
         <v>195</v>
       </c>
-      <c r="I30" t="s">
-        <v>74</v>
+      <c r="I30" s="12" t="s">
+        <v>255</v>
       </c>
       <c r="P30" t="s">
         <v>249</v>
@@ -4879,13 +4889,13 @@
         <v>252</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="F31" t="s">
         <v>195</v>
       </c>
-      <c r="I31" t="s">
-        <v>74</v>
+      <c r="I31" s="12" t="s">
+        <v>255</v>
       </c>
       <c r="P31" t="s">
         <v>249</v>
@@ -4899,7 +4909,7 @@
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D32" t="s">
         <v>253</v>
@@ -4910,7 +4920,7 @@
       <c r="F32" t="s">
         <v>195</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="12" t="s">
         <v>255</v>
       </c>
     </row>
@@ -4919,7 +4929,7 @@
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D33" t="s">
         <v>256</v>
@@ -4931,7 +4941,7 @@
         <v>195</v>
       </c>
       <c r="I33" t="s">
-        <v>258</v>
+        <v>203</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
@@ -4939,7 +4949,7 @@
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D34" t="s">
         <v>259</v>
@@ -4959,7 +4969,7 @@
         <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D35" t="s">
         <v>261</v>
@@ -4979,7 +4989,7 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D36" t="s">
         <v>263</v>
@@ -4991,7 +5001,7 @@
         <v>195</v>
       </c>
       <c r="I36" t="s">
-        <v>255</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.35">
@@ -4999,7 +5009,7 @@
         <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D37" t="s">
         <v>265</v>
@@ -5031,7 +5041,7 @@
         <v>195</v>
       </c>
       <c r="I38" t="s">
-        <v>255</v>
+        <v>203</v>
       </c>
       <c r="P38" t="s">
         <v>269</v>
@@ -5088,19 +5098,19 @@
         <v>5</v>
       </c>
       <c r="C41" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="D41" t="s">
         <v>379</v>
       </c>
-      <c r="D41" t="s">
-        <v>380</v>
-      </c>
       <c r="E41" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F41" t="s">
         <v>195</v>
       </c>
-      <c r="I41" t="s">
-        <v>255</v>
+      <c r="I41" s="12" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.35">
@@ -5170,8 +5180,8 @@
       <c r="F45" t="s">
         <v>195</v>
       </c>
-      <c r="I45" t="s">
-        <v>6</v>
+      <c r="I45" s="12" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.35">
@@ -5190,7 +5200,7 @@
       <c r="F46" t="s">
         <v>195</v>
       </c>
-      <c r="I46" t="s">
+      <c r="I46" s="12" t="s">
         <v>74</v>
       </c>
     </row>
@@ -5239,6 +5249,9 @@
       <c r="G48" t="s">
         <v>291</v>
       </c>
+      <c r="I48" s="12" t="s">
+        <v>109</v>
+      </c>
       <c r="J48" t="s">
         <v>287</v>
       </c>
@@ -5385,36 +5398,42 @@
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>6</v>
+      </c>
       <c r="C55" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F55" t="s">
         <v>195</v>
       </c>
-      <c r="I55" t="s">
+      <c r="I55" s="12" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>6</v>
+      </c>
       <c r="C56" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F56" t="s">
         <v>195</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I56" s="12" t="s">
         <v>255</v>
       </c>
     </row>
@@ -5429,13 +5448,13 @@
         <v>310</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F57" t="s">
         <v>195</v>
       </c>
-      <c r="I57" t="s">
-        <v>311</v>
+      <c r="I57" s="12" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.35">
@@ -5443,19 +5462,19 @@
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F58" t="s">
         <v>195</v>
       </c>
-      <c r="I58" t="s">
-        <v>109</v>
+      <c r="I58" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="P58" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.35">
@@ -5463,19 +5482,19 @@
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F59" t="s">
         <v>195</v>
       </c>
-      <c r="I59" t="s">
-        <v>109</v>
+      <c r="I59" s="12" t="s">
+        <v>74</v>
       </c>
       <c r="P59" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.35">
@@ -5483,19 +5502,19 @@
         <v>8</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D60" t="s">
         <v>315</v>
       </c>
-      <c r="D60" t="s">
-        <v>316</v>
-      </c>
       <c r="E60" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F60" t="s">
         <v>195</v>
       </c>
       <c r="I60" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.35">
@@ -5503,19 +5522,19 @@
         <v>9</v>
       </c>
       <c r="B61" t="s">
+        <v>317</v>
+      </c>
+      <c r="D61" t="s">
         <v>318</v>
       </c>
-      <c r="D61" t="s">
-        <v>319</v>
-      </c>
       <c r="E61" s="6" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F61" t="s">
         <v>195</v>
       </c>
       <c r="I61" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.35">
@@ -5523,10 +5542,10 @@
         <v>9</v>
       </c>
       <c r="D62" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E62" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F62" t="s">
         <v>195</v>
@@ -5537,13 +5556,13 @@
         <v>9</v>
       </c>
       <c r="D63" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E63" t="s">
+        <v>372</v>
+      </c>
+      <c r="F63" t="s">
         <v>373</v>
-      </c>
-      <c r="F63" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.35">
@@ -5551,16 +5570,16 @@
         <v>9</v>
       </c>
       <c r="D64" t="s">
+        <v>320</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>322</v>
       </c>
       <c r="F64" t="s">
         <v>195</v>
       </c>
       <c r="I64" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.35">
@@ -5568,16 +5587,16 @@
         <v>9</v>
       </c>
       <c r="D65" t="s">
+        <v>323</v>
+      </c>
+      <c r="E65" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="F65" t="s">
         <v>325</v>
       </c>
-      <c r="F65" t="s">
+      <c r="O65" t="s">
         <v>326</v>
-      </c>
-      <c r="O65" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.35">
@@ -5585,13 +5604,13 @@
         <v>3</v>
       </c>
       <c r="B66" t="s">
+        <v>327</v>
+      </c>
+      <c r="D66" t="s">
         <v>328</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>329</v>
-      </c>
-      <c r="E66" t="s">
-        <v>330</v>
       </c>
       <c r="F66" t="s">
         <v>195</v>
@@ -5605,19 +5624,19 @@
         <v>3</v>
       </c>
       <c r="D67" t="s">
+        <v>330</v>
+      </c>
+      <c r="E67" t="s">
         <v>331</v>
-      </c>
-      <c r="E67" t="s">
-        <v>332</v>
       </c>
       <c r="F67" t="s">
         <v>195</v>
       </c>
       <c r="G67" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="I67" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.35">
@@ -5625,19 +5644,19 @@
         <v>3</v>
       </c>
       <c r="D68" t="s">
+        <v>333</v>
+      </c>
+      <c r="E68" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>335</v>
       </c>
       <c r="F68" t="s">
         <v>195</v>
       </c>
       <c r="G68" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="I68" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.35">
@@ -5645,13 +5664,13 @@
         <v>10</v>
       </c>
       <c r="B69" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="D69" t="s">
         <v>336</v>
       </c>
-      <c r="D69" t="s">
+      <c r="F69" t="s">
         <v>337</v>
-      </c>
-      <c r="F69" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.35">
@@ -5659,10 +5678,10 @@
         <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F70" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.35">
@@ -5670,10 +5689,10 @@
         <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F71" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.35">
@@ -5681,10 +5700,10 @@
         <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F72" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.35">
@@ -5692,10 +5711,10 @@
         <v>10</v>
       </c>
       <c r="D73" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F73" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.35">
@@ -5703,22 +5722,22 @@
         <v>5</v>
       </c>
       <c r="C74" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D74" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F74" t="s">
         <v>195</v>
       </c>
       <c r="I74" t="s">
-        <v>255</v>
+        <v>203</v>
       </c>
       <c r="P74" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.35">
@@ -5726,42 +5745,42 @@
         <v>5</v>
       </c>
       <c r="C75" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D75" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F75" t="s">
         <v>195</v>
       </c>
-      <c r="I75" t="s">
+      <c r="I75" s="12" t="s">
         <v>255</v>
       </c>
       <c r="P75" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A76" s="6">
+      <c r="A76" s="13">
         <v>5</v>
       </c>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6" t="s">
-        <v>359</v>
-      </c>
-      <c r="D76" s="6" t="s">
+      <c r="B76" s="13"/>
+      <c r="C76" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="D76" s="13" t="s">
+        <v>345</v>
+      </c>
+      <c r="E76" s="13" t="s">
         <v>346</v>
       </c>
-      <c r="E76" s="6" t="s">
-        <v>347</v>
-      </c>
-      <c r="F76" s="6" t="s">
+      <c r="F76" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="I76" t="s">
+      <c r="I76" s="13" t="s">
         <v>74</v>
       </c>
     </row>
@@ -5780,24 +5799,24 @@
         <v>179</v>
       </c>
       <c r="B1" t="s">
+        <v>380</v>
+      </c>
+      <c r="C1" t="s">
         <v>381</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>382</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>383</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>384</v>
-      </c>
-      <c r="F1" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -5811,7 +5830,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C3">
         <v>60</v>
@@ -5825,7 +5844,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C4">
         <v>90</v>
@@ -5839,7 +5858,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C5">
         <v>120</v>
@@ -5853,7 +5872,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C6">
         <v>180</v>
@@ -5867,7 +5886,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C7">
         <v>240</v>
@@ -5881,7 +5900,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C8">
         <v>30</v>
@@ -5895,7 +5914,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C9">
         <v>60</v>
@@ -5909,7 +5928,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C10">
         <v>90</v>
@@ -5923,7 +5942,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C11">
         <v>120</v>
@@ -5937,7 +5956,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C12">
         <v>180</v>
@@ -5951,7 +5970,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C13">
         <v>240</v>
@@ -5965,7 +5984,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C14">
         <v>60</v>
@@ -5979,7 +5998,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C15">
         <v>90</v>
@@ -5993,7 +6012,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C16">
         <v>120</v>
@@ -6007,10 +6026,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>388</v>
+      </c>
+      <c r="B17" t="s">
         <v>389</v>
-      </c>
-      <c r="B17" t="s">
-        <v>390</v>
       </c>
       <c r="C17">
         <v>60</v>
@@ -6021,10 +6040,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B18" t="s">
         <v>389</v>
-      </c>
-      <c r="B18" t="s">
-        <v>390</v>
       </c>
       <c r="C18">
         <v>120</v>
@@ -6035,10 +6054,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B19" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C19">
         <v>30</v>
@@ -6049,10 +6068,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B20" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C20">
         <v>90</v>

</xml_diff>

<commit_message>
Updated apparatus list. (removed hose reels cabinets & valves, removed sprinkler & hydrant pumps, added pumpsets)
</commit_message>
<xml_diff>
--- a/database/databases/Standards_Calc_Database_Finalised.xlsx
+++ b/database/databases/Standards_Calc_Database_Finalised.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\JFC-Embodied-Carbon-App\database\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BABC4F-4E5B-42D8-A082-9B6033764322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53A83EC-F070-4258-9E69-E55BD2213754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1128" uniqueCount="382">
   <si>
     <t>system</t>
   </si>
@@ -763,18 +763,6 @@
     <t>Pipework</t>
   </si>
   <si>
-    <t>Hose Reel Cabinets</t>
-  </si>
-  <si>
-    <t>Cabinet</t>
-  </si>
-  <si>
-    <t>Hose Reel Valves</t>
-  </si>
-  <si>
-    <t>Valve</t>
-  </si>
-  <si>
     <t>Means of Restricting Fire Spread / Structural Protection</t>
   </si>
   <si>
@@ -925,15 +913,6 @@
     <t>Sprinkler Valve</t>
   </si>
   <si>
-    <t>Sprinkler Pumps</t>
-  </si>
-  <si>
-    <t>Sprinkler Pump</t>
-  </si>
-  <si>
-    <t>pumps</t>
-  </si>
-  <si>
     <t>Hydrants</t>
   </si>
   <si>
@@ -958,12 +937,6 @@
     <t>Typically 1 booster assembly per hydrant system - confirm against site layout and AS2419.1.</t>
   </si>
   <si>
-    <t>Hydrant Pumps</t>
-  </si>
-  <si>
-    <t>Hydrant Pump</t>
-  </si>
-  <si>
     <t>Means of Smoke Hazard Management</t>
   </si>
   <si>
@@ -989,9 +962,6 @@
   </si>
   <si>
     <t>Fire Safety Management</t>
-  </si>
-  <si>
-    <t>Fire Safety Signage</t>
   </si>
   <si>
     <t>signs</t>
@@ -1217,16 +1187,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1238,7 +1202,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1254,12 +1218,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1306,21 +1264,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4160,7 +4115,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="17" width="20" customWidth="1"/>
@@ -4219,11 +4174,11 @@
         <v>191</v>
       </c>
       <c r="R1" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="9">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -4319,8 +4274,8 @@
       <c r="F5" t="s">
         <v>195</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>255</v>
+      <c r="I5" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
@@ -4351,7 +4306,7 @@
         <v>206</v>
       </c>
       <c r="E7" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="F7" t="s">
         <v>195</v>
@@ -4378,7 +4333,7 @@
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A9" s="9">
+      <c r="A9" s="7">
         <v>2</v>
       </c>
       <c r="B9" t="s">
@@ -4582,8 +4537,8 @@
       <c r="D18" t="s">
         <v>230</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>364</v>
+      <c r="E18" s="7" t="s">
+        <v>354</v>
       </c>
       <c r="F18" t="s">
         <v>195</v>
@@ -4625,8 +4580,8 @@
       <c r="D20" t="s">
         <v>232</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>365</v>
+      <c r="E20" s="7" t="s">
+        <v>355</v>
       </c>
       <c r="F20" t="s">
         <v>195</v>
@@ -4682,7 +4637,7 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A23" s="9">
+      <c r="A23" s="7">
         <v>4</v>
       </c>
       <c r="B23" t="s">
@@ -4695,7 +4650,7 @@
         <v>238</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="F23" t="s">
         <v>195</v>
@@ -4725,105 +4680,111 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A25">
+      <c r="A25" s="3">
         <v>4</v>
       </c>
-      <c r="C25" t="s">
-        <v>237</v>
-      </c>
-      <c r="D25" t="s">
-        <v>242</v>
+      <c r="B25" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>339</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="F25" t="s">
-        <v>216</v>
-      </c>
-      <c r="J25" t="s">
-        <v>238</v>
-      </c>
-      <c r="K25" t="s">
-        <v>226</v>
-      </c>
+        <v>340</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B26" t="s">
+        <v>242</v>
       </c>
       <c r="C26" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D26" t="s">
         <v>244</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="F26" t="s">
+        <v>195</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="P26" t="s">
         <v>245</v>
       </c>
-      <c r="F26" t="s">
-        <v>216</v>
-      </c>
-      <c r="J26" t="s">
-        <v>238</v>
-      </c>
-      <c r="K26" t="s">
-        <v>226</v>
+      <c r="R26" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A27" s="4">
-        <v>4</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="F27" s="4" t="s">
+      <c r="A27">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>243</v>
+      </c>
+      <c r="D27" t="s">
+        <v>246</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F27" t="s">
         <v>195</v>
       </c>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="I27" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="P27" t="s">
+        <v>245</v>
+      </c>
+      <c r="R27" t="s">
+        <v>285</v>
+      </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>5</v>
       </c>
-      <c r="B28" t="s">
-        <v>246</v>
-      </c>
       <c r="C28" t="s">
+        <v>243</v>
+      </c>
+      <c r="D28" t="s">
         <v>247</v>
       </c>
-      <c r="D28" t="s">
-        <v>248</v>
-      </c>
       <c r="E28" s="1" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="F28" t="s">
         <v>195</v>
       </c>
-      <c r="I28" s="12" t="s">
-        <v>74</v>
+      <c r="I28" s="10" t="s">
+        <v>251</v>
       </c>
       <c r="P28" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="R28" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
@@ -4831,25 +4792,25 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D29" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="F29" t="s">
         <v>195</v>
       </c>
-      <c r="I29" s="12" t="s">
-        <v>255</v>
+      <c r="I29" s="10" t="s">
+        <v>251</v>
       </c>
       <c r="P29" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="R29" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
@@ -4857,25 +4818,19 @@
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>247</v>
+        <v>345</v>
       </c>
       <c r="D30" t="s">
-        <v>251</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>353</v>
+        <v>249</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>250</v>
       </c>
       <c r="F30" t="s">
         <v>195</v>
       </c>
-      <c r="I30" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="P30" t="s">
-        <v>249</v>
-      </c>
-      <c r="R30" t="s">
-        <v>289</v>
+      <c r="I30" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
@@ -4883,25 +4838,19 @@
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>247</v>
+        <v>346</v>
       </c>
       <c r="D31" t="s">
         <v>252</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>354</v>
+      <c r="E31" s="4" t="s">
+        <v>253</v>
       </c>
       <c r="F31" t="s">
         <v>195</v>
       </c>
-      <c r="I31" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="P31" t="s">
-        <v>249</v>
-      </c>
-      <c r="R31" t="s">
-        <v>289</v>
+      <c r="I31" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
@@ -4909,19 +4858,19 @@
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="D32" t="s">
-        <v>253</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>256</v>
       </c>
       <c r="F32" t="s">
         <v>195</v>
       </c>
-      <c r="I32" s="12" t="s">
-        <v>255</v>
+      <c r="I32" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.35">
@@ -4929,19 +4878,19 @@
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="D33" t="s">
-        <v>256</v>
-      </c>
-      <c r="E33" s="5" t="s">
         <v>257</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>258</v>
       </c>
       <c r="F33" t="s">
         <v>195</v>
       </c>
       <c r="I33" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
@@ -4949,19 +4898,19 @@
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="D34" t="s">
         <v>259</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="4" t="s">
         <v>260</v>
       </c>
       <c r="F34" t="s">
         <v>195</v>
       </c>
       <c r="I34" t="s">
-        <v>258</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.35">
@@ -4969,19 +4918,19 @@
         <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="D35" t="s">
         <v>261</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F35" t="s">
         <v>195</v>
       </c>
       <c r="I35" t="s">
-        <v>258</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.35">
@@ -4989,12 +4938,12 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>358</v>
+        <v>262</v>
       </c>
       <c r="D36" t="s">
         <v>263</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E36" s="4" t="s">
         <v>264</v>
       </c>
       <c r="F36" t="s">
@@ -5002,6 +4951,9 @@
       </c>
       <c r="I36" t="s">
         <v>203</v>
+      </c>
+      <c r="P36" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.35">
@@ -5009,19 +4961,22 @@
         <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>358</v>
+        <v>262</v>
       </c>
       <c r="D37" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F37" t="s">
         <v>195</v>
       </c>
       <c r="I37" t="s">
-        <v>74</v>
+        <v>268</v>
+      </c>
+      <c r="P37" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.35">
@@ -5029,88 +4984,76 @@
         <v>5</v>
       </c>
       <c r="C38" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D38" t="s">
-        <v>267</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>271</v>
       </c>
       <c r="F38" t="s">
         <v>195</v>
       </c>
       <c r="I38" t="s">
-        <v>203</v>
+        <v>109</v>
       </c>
       <c r="P38" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>5</v>
       </c>
-      <c r="C39" t="s">
-        <v>266</v>
+      <c r="C39" s="8" t="s">
+        <v>368</v>
       </c>
       <c r="D39" t="s">
-        <v>270</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>271</v>
+        <v>369</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>369</v>
       </c>
       <c r="F39" t="s">
         <v>195</v>
       </c>
-      <c r="I39" t="s">
-        <v>272</v>
-      </c>
-      <c r="P39" t="s">
-        <v>273</v>
+      <c r="I39" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>5</v>
       </c>
-      <c r="C40" t="s">
-        <v>266</v>
-      </c>
       <c r="D40" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F40" t="s">
         <v>195</v>
       </c>
       <c r="I40" t="s">
-        <v>109</v>
-      </c>
-      <c r="P40" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>5</v>
       </c>
-      <c r="C41" s="10" t="s">
-        <v>378</v>
-      </c>
       <c r="D41" t="s">
-        <v>379</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>379</v>
+        <v>275</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>275</v>
       </c>
       <c r="F41" t="s">
         <v>195</v>
       </c>
-      <c r="I41" s="12" t="s">
-        <v>74</v>
+      <c r="I41" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.35">
@@ -5118,154 +5061,166 @@
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F42" t="s">
         <v>195</v>
       </c>
       <c r="I42" t="s">
-        <v>278</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>5</v>
       </c>
+      <c r="C43" t="s">
+        <v>278</v>
+      </c>
       <c r="D43" t="s">
-        <v>279</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>278</v>
       </c>
       <c r="F43" t="s">
         <v>195</v>
       </c>
-      <c r="I43" t="s">
-        <v>278</v>
+      <c r="I43" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>5</v>
       </c>
+      <c r="C44" t="s">
+        <v>280</v>
+      </c>
       <c r="D44" t="s">
-        <v>280</v>
-      </c>
-      <c r="E44" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E44" s="4" t="s">
         <v>280</v>
       </c>
       <c r="F44" t="s">
         <v>195</v>
       </c>
-      <c r="I44" t="s">
+      <c r="I44" s="10" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A45">
-        <v>5</v>
+      <c r="A45" s="7">
+        <v>6</v>
+      </c>
+      <c r="B45" t="s">
+        <v>281</v>
       </c>
       <c r="C45" t="s">
         <v>282</v>
       </c>
       <c r="D45" t="s">
-        <v>281</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>282</v>
+        <v>283</v>
+      </c>
+      <c r="E45" t="s">
+        <v>284</v>
       </c>
       <c r="F45" t="s">
         <v>195</v>
       </c>
-      <c r="I45" s="12" t="s">
-        <v>74</v>
+      <c r="G45" t="s">
+        <v>213</v>
+      </c>
+      <c r="H45" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D46" t="s">
-        <v>283</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>284</v>
+        <v>286</v>
+      </c>
+      <c r="E46" t="s">
+        <v>286</v>
       </c>
       <c r="F46" t="s">
         <v>195</v>
       </c>
-      <c r="I46" s="12" t="s">
-        <v>74</v>
+      <c r="G46" t="s">
+        <v>287</v>
+      </c>
+      <c r="I46" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="J46" t="s">
+        <v>283</v>
+      </c>
+      <c r="L46" t="s">
+        <v>8</v>
+      </c>
+      <c r="M46" t="s">
+        <v>22</v>
+      </c>
+      <c r="N46" t="s">
+        <v>288</v>
+      </c>
+      <c r="P46" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A47" s="9">
+      <c r="A47">
         <v>6</v>
       </c>
-      <c r="B47" t="s">
-        <v>285</v>
-      </c>
       <c r="C47" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="D47" t="s">
-        <v>287</v>
-      </c>
-      <c r="E47" t="s">
-        <v>288</v>
+        <v>290</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>291</v>
       </c>
       <c r="F47" t="s">
-        <v>195</v>
-      </c>
-      <c r="G47" t="s">
-        <v>213</v>
-      </c>
-      <c r="H47" t="s">
-        <v>289</v>
+        <v>216</v>
+      </c>
+      <c r="J47" t="s">
+        <v>283</v>
+      </c>
+      <c r="K47" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>6</v>
       </c>
-      <c r="C48" t="s">
-        <v>286</v>
-      </c>
-      <c r="D48" t="s">
-        <v>290</v>
-      </c>
-      <c r="E48" t="s">
-        <v>290</v>
+      <c r="C48" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>292</v>
       </c>
       <c r="F48" t="s">
         <v>195</v>
       </c>
-      <c r="G48" t="s">
-        <v>291</v>
-      </c>
-      <c r="I48" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="J48" t="s">
-        <v>287</v>
-      </c>
-      <c r="L48" t="s">
-        <v>8</v>
-      </c>
-      <c r="M48" t="s">
-        <v>22</v>
-      </c>
-      <c r="N48" t="s">
-        <v>292</v>
+      <c r="I48" t="s">
+        <v>293</v>
       </c>
       <c r="P48" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.35">
@@ -5273,22 +5228,19 @@
         <v>6</v>
       </c>
       <c r="C49" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D49" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>295</v>
       </c>
       <c r="F49" t="s">
-        <v>216</v>
-      </c>
-      <c r="J49" t="s">
-        <v>287</v>
-      </c>
-      <c r="K49" t="s">
-        <v>226</v>
+        <v>195</v>
+      </c>
+      <c r="I49" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.35">
@@ -5296,12 +5248,12 @@
         <v>6</v>
       </c>
       <c r="C50" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D50" t="s">
         <v>296</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="E50" s="2" t="s">
         <v>297</v>
       </c>
       <c r="F50" t="s">
@@ -5309,217 +5261,199 @@
       </c>
       <c r="I50" t="s">
         <v>298</v>
+      </c>
+      <c r="P50" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>6</v>
       </c>
-      <c r="C51" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>299</v>
+      <c r="C51" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>358</v>
       </c>
       <c r="F51" t="s">
         <v>195</v>
       </c>
-      <c r="I51" t="s">
-        <v>300</v>
-      </c>
-      <c r="P51" t="s">
-        <v>301</v>
+      <c r="I51" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>6</v>
       </c>
-      <c r="C52" t="s">
-        <v>299</v>
-      </c>
-      <c r="D52" t="s">
-        <v>302</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>302</v>
+      <c r="C52" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>357</v>
       </c>
       <c r="F52" t="s">
         <v>195</v>
       </c>
-      <c r="I52" t="s">
-        <v>109</v>
+      <c r="I52" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A53">
-        <v>6</v>
-      </c>
-      <c r="C53" t="s">
-        <v>299</v>
+      <c r="A53" s="7">
+        <v>7</v>
+      </c>
+      <c r="B53" t="s">
+        <v>300</v>
       </c>
       <c r="D53" t="s">
-        <v>303</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>350</v>
       </c>
       <c r="F53" t="s">
         <v>195</v>
       </c>
-      <c r="I53" t="s">
-        <v>305</v>
-      </c>
-      <c r="P53" t="s">
-        <v>306</v>
+      <c r="I53" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54">
-        <v>6</v>
-      </c>
-      <c r="C54" t="s">
-        <v>299</v>
+        <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>307</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>308</v>
+        <v>302</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>353</v>
       </c>
       <c r="F54" t="s">
         <v>195</v>
       </c>
-      <c r="I54" t="s">
-        <v>298</v>
+      <c r="I54" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="P54" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55">
-        <v>6</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>359</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>369</v>
-      </c>
-      <c r="E55" s="11" t="s">
-        <v>368</v>
+        <v>7</v>
+      </c>
+      <c r="D55" t="s">
+        <v>304</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>352</v>
       </c>
       <c r="F55" t="s">
         <v>195</v>
       </c>
-      <c r="I55" s="12" t="s">
-        <v>255</v>
+      <c r="I55" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="P55" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A56">
-        <v>6</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>359</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>370</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>367</v>
+      <c r="A56" s="7">
+        <v>8</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D56" t="s">
+        <v>306</v>
+      </c>
+      <c r="E56" t="s">
+        <v>306</v>
       </c>
       <c r="F56" t="s">
         <v>195</v>
       </c>
-      <c r="I56" s="12" t="s">
-        <v>255</v>
+      <c r="I56" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A57" s="9">
-        <v>7</v>
+      <c r="A57" s="7">
+        <v>9</v>
       </c>
       <c r="B57" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D57" t="s">
-        <v>310</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>360</v>
+        <v>364</v>
+      </c>
+      <c r="E57" t="s">
+        <v>361</v>
       </c>
       <c r="F57" t="s">
         <v>195</v>
       </c>
-      <c r="I57" s="12" t="s">
-        <v>255</v>
-      </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A58">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D58" t="s">
-        <v>311</v>
-      </c>
-      <c r="E58" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="E58" t="s">
+        <v>362</v>
+      </c>
+      <c r="F58" t="s">
         <v>363</v>
-      </c>
-      <c r="F58" t="s">
-        <v>195</v>
-      </c>
-      <c r="I58" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="P58" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A59">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D59" t="s">
-        <v>313</v>
-      </c>
-      <c r="E59" s="9" t="s">
-        <v>362</v>
+        <v>310</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>311</v>
       </c>
       <c r="F59" t="s">
         <v>195</v>
       </c>
-      <c r="I59" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="P59" t="s">
+      <c r="I59" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A60" s="9">
-        <v>8</v>
-      </c>
-      <c r="B60" s="2" t="s">
+      <c r="A60">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>313</v>
+      </c>
+      <c r="E60" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="D60" t="s">
+      <c r="F60" t="s">
         <v>315</v>
       </c>
-      <c r="E60" t="s">
-        <v>315</v>
-      </c>
-      <c r="F60" t="s">
-        <v>195</v>
-      </c>
-      <c r="I60" t="s">
+      <c r="O60" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A61" s="9">
-        <v>9</v>
+      <c r="A61" s="7">
+        <v>3</v>
       </c>
       <c r="B61" t="s">
         <v>317</v>
@@ -5527,260 +5461,177 @@
       <c r="D61" t="s">
         <v>318</v>
       </c>
-      <c r="E61" s="6" t="s">
-        <v>318</v>
+      <c r="E61" t="s">
+        <v>319</v>
       </c>
       <c r="F61" t="s">
         <v>195</v>
       </c>
-      <c r="I61" t="s">
-        <v>319</v>
+      <c r="G61" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D62" t="s">
-        <v>374</v>
+        <v>320</v>
       </c>
       <c r="E62" t="s">
-        <v>371</v>
+        <v>321</v>
       </c>
       <c r="F62" t="s">
         <v>195</v>
       </c>
+      <c r="G62" t="s">
+        <v>322</v>
+      </c>
+      <c r="I62" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D63" t="s">
-        <v>375</v>
-      </c>
-      <c r="E63" t="s">
-        <v>372</v>
+        <v>323</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>324</v>
       </c>
       <c r="F63" t="s">
-        <v>373</v>
+        <v>195</v>
+      </c>
+      <c r="G63" t="s">
+        <v>322</v>
+      </c>
+      <c r="I63" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A64">
-        <v>9</v>
+      <c r="A64" s="7">
+        <v>10</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>325</v>
       </c>
       <c r="D64" t="s">
-        <v>320</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="F64" t="s">
-        <v>195</v>
-      </c>
-      <c r="I64" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D65" t="s">
-        <v>323</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="F65" t="s">
-        <v>325</v>
-      </c>
-      <c r="O65" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A66" s="9">
-        <v>3</v>
-      </c>
-      <c r="B66" t="s">
+      <c r="A66">
+        <v>10</v>
+      </c>
+      <c r="D66" t="s">
+        <v>329</v>
+      </c>
+      <c r="F66" t="s">
         <v>327</v>
-      </c>
-      <c r="D66" t="s">
-        <v>328</v>
-      </c>
-      <c r="E66" t="s">
-        <v>329</v>
-      </c>
-      <c r="F66" t="s">
-        <v>195</v>
-      </c>
-      <c r="G66" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D67" t="s">
         <v>330</v>
       </c>
-      <c r="E67" t="s">
-        <v>331</v>
-      </c>
       <c r="F67" t="s">
-        <v>195</v>
-      </c>
-      <c r="G67" t="s">
-        <v>332</v>
-      </c>
-      <c r="I67" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A68">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D68" t="s">
+        <v>331</v>
+      </c>
+      <c r="F68" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>5</v>
+      </c>
+      <c r="C69" t="s">
+        <v>351</v>
+      </c>
+      <c r="D69" t="s">
+        <v>366</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="F69" t="s">
+        <v>195</v>
+      </c>
+      <c r="I69" t="s">
+        <v>203</v>
+      </c>
+      <c r="P69" t="s">
         <v>333</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="F68" t="s">
-        <v>195</v>
-      </c>
-      <c r="G68" t="s">
-        <v>332</v>
-      </c>
-      <c r="I68" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A69" s="9">
-        <v>10</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="D69" t="s">
-        <v>336</v>
-      </c>
-      <c r="F69" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A70">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="C70" t="s">
+        <v>351</v>
       </c>
       <c r="D70" t="s">
-        <v>338</v>
+        <v>367</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>334</v>
       </c>
       <c r="F70" t="s">
-        <v>337</v>
+        <v>195</v>
+      </c>
+      <c r="I70" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="P70" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A71">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="C71" t="s">
+        <v>347</v>
       </c>
       <c r="D71" t="s">
-        <v>339</v>
+        <v>335</v>
+      </c>
+      <c r="E71" t="s">
+        <v>336</v>
       </c>
       <c r="F71" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A72">
-        <v>10</v>
-      </c>
-      <c r="D72" t="s">
-        <v>340</v>
-      </c>
-      <c r="F72" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A73">
-        <v>10</v>
-      </c>
-      <c r="D73" t="s">
-        <v>341</v>
-      </c>
-      <c r="F73" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A74">
-        <v>5</v>
-      </c>
-      <c r="C74" t="s">
-        <v>361</v>
-      </c>
-      <c r="D74" t="s">
-        <v>376</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="F74" t="s">
         <v>195</v>
       </c>
-      <c r="I74" t="s">
-        <v>203</v>
-      </c>
-      <c r="P74" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A75">
-        <v>5</v>
-      </c>
-      <c r="C75" t="s">
-        <v>361</v>
-      </c>
-      <c r="D75" t="s">
-        <v>377</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="F75" t="s">
-        <v>195</v>
-      </c>
-      <c r="I75" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="P75" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A76" s="13">
-        <v>5</v>
-      </c>
-      <c r="B76" s="13"/>
-      <c r="C76" s="13" t="s">
-        <v>357</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>345</v>
-      </c>
-      <c r="E76" s="13" t="s">
-        <v>346</v>
-      </c>
-      <c r="F76" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="I76" s="13" t="s">
+      <c r="I71" t="s">
         <v>74</v>
       </c>
     </row>
@@ -5799,24 +5650,24 @@
         <v>179</v>
       </c>
       <c r="B1" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="D1" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="E1" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="F1" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -5830,7 +5681,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C3">
         <v>60</v>
@@ -5844,7 +5695,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C4">
         <v>90</v>
@@ -5858,7 +5709,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C5">
         <v>120</v>
@@ -5872,7 +5723,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C6">
         <v>180</v>
@@ -5886,7 +5737,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="C7">
         <v>240</v>
@@ -5900,7 +5751,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C8">
         <v>30</v>
@@ -5914,7 +5765,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C9">
         <v>60</v>
@@ -5928,7 +5779,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C10">
         <v>90</v>
@@ -5942,7 +5793,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C11">
         <v>120</v>
@@ -5956,7 +5807,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C12">
         <v>180</v>
@@ -5970,7 +5821,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="C13">
         <v>240</v>
@@ -5984,7 +5835,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="C14">
         <v>60</v>
@@ -5998,7 +5849,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="C15">
         <v>90</v>
@@ -6012,7 +5863,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="C16">
         <v>120</v>
@@ -6026,10 +5877,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="B17" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="C17">
         <v>60</v>
@@ -6040,10 +5891,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="B18" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="C18">
         <v>120</v>
@@ -6054,10 +5905,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="B19" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C19">
         <v>30</v>
@@ -6068,10 +5919,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="B20" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C20">
         <v>90</v>

</xml_diff>

<commit_message>
database units edit 2.0
</commit_message>
<xml_diff>
--- a/database/databases/Standards_Calc_Database_Finalised.xlsx
+++ b/database/databases/Standards_Calc_Database_Finalised.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\JFC-Embodied-Carbon-App\database\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53A83EC-F070-4258-9E69-E55BD2213754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39AFB3E-7675-41F9-A01C-C96ACD46C40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4752,7 +4752,7 @@
         <v>195</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>251</v>
+        <v>74</v>
       </c>
       <c r="P27" t="s">
         <v>245</v>
@@ -4778,7 +4778,7 @@
         <v>195</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>251</v>
+        <v>74</v>
       </c>
       <c r="P28" t="s">
         <v>245</v>
@@ -4804,7 +4804,7 @@
         <v>195</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>251</v>
+        <v>74</v>
       </c>
       <c r="P29" t="s">
         <v>245</v>
@@ -5644,6 +5644,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9B6005-6F43-4EB4-8661-C70A2093261E}">
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.6328125" customWidth="1"/>
+    <col min="2" max="7" width="13.6328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
Building inputs autoloads when looking at past projects
</commit_message>
<xml_diff>
--- a/database/databases/Standards_Calc_Database_Finalised.xlsx
+++ b/database/databases/Standards_Calc_Database_Finalised.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\JFC\04_Software\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\JFC-Embodied-Carbon-App\database\databases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADFC0594-0FAF-4F96-9C6F-90C20928A5AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7138E96E-2F5F-463F-811E-A68081B52E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="385">
   <si>
     <t>Category</t>
   </si>
@@ -608,9 +608,6 @@
   </si>
   <si>
     <t>Fire Equipment Identification Sign</t>
-  </si>
-  <si>
-    <t>Cross-Category Counter</t>
   </si>
   <si>
     <t>Extinguishers,Hose Reel Assembly,Hydrants,Hydrant Boosters</t>
@@ -1202,7 +1199,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1736,17 +1733,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AR102"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="17" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:31" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1802,7 +1799,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="18" customFormat="1">
+    <row r="2" spans="1:31" s="18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="16">
         <v>1</v>
       </c>
@@ -1840,7 +1837,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:31">
+    <row r="3" spans="1:31" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="17">
         <v>1</v>
       </c>
@@ -1878,7 +1875,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:31">
+    <row r="4" spans="1:31" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="17">
         <v>1</v>
       </c>
@@ -1901,7 +1898,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:31">
+    <row r="5" spans="1:31" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="17">
         <v>1</v>
       </c>
@@ -1924,7 +1921,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:31" s="5" customFormat="1">
+    <row r="6" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="11">
         <v>1</v>
       </c>
@@ -1945,7 +1942,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:31" s="5" customFormat="1">
+    <row r="7" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
         <v>1</v>
       </c>
@@ -1966,7 +1963,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="5" customFormat="1">
+    <row r="8" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="11">
         <v>1</v>
       </c>
@@ -1990,7 +1987,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="5" customFormat="1">
+    <row r="9" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
         <v>1</v>
       </c>
@@ -2011,7 +2008,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="5" customFormat="1">
+    <row r="10" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="11">
         <v>1</v>
       </c>
@@ -2032,7 +2029,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:31">
+    <row r="11" spans="1:31" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="17">
         <v>1</v>
       </c>
@@ -2067,7 +2064,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:31" s="5" customFormat="1">
+    <row r="12" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" s="17">
         <v>1</v>
       </c>
@@ -2114,7 +2111,7 @@
       <c r="AD12" s="12"/>
       <c r="AE12" s="12"/>
     </row>
-    <row r="13" spans="1:31" s="5" customFormat="1">
+    <row r="13" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
         <v>1</v>
       </c>
@@ -2138,7 +2135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="5" customFormat="1">
+    <row r="14" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="11">
         <v>1</v>
       </c>
@@ -2162,7 +2159,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="5" customFormat="1">
+    <row r="15" spans="1:31" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="11">
         <v>1</v>
       </c>
@@ -2186,7 +2183,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:31" s="22" customFormat="1">
+    <row r="16" spans="1:31" s="22" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <v>1</v>
       </c>
@@ -2211,7 +2208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="25">
         <v>2</v>
       </c>
@@ -2234,7 +2231,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:18" s="1" customFormat="1">
+    <row r="18" spans="1:18" s="1" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A18" s="25">
         <v>2</v>
       </c>
@@ -2263,7 +2260,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:18" s="5" customFormat="1">
+    <row r="19" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A19" s="25">
         <v>2</v>
       </c>
@@ -2283,7 +2280,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:18" s="18" customFormat="1">
+    <row r="20" spans="1:18" s="18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="24">
         <v>2</v>
       </c>
@@ -2309,7 +2306,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:18" s="5" customFormat="1">
+    <row r="21" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="45">
         <v>2</v>
       </c>
@@ -2332,7 +2329,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:18" s="5" customFormat="1">
+    <row r="22" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="25">
         <v>2</v>
       </c>
@@ -2361,7 +2358,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:18" s="22" customFormat="1">
+    <row r="23" spans="1:18" s="22" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="26">
         <v>2</v>
       </c>
@@ -2385,7 +2382,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="17">
         <v>3</v>
       </c>
@@ -2411,7 +2408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:18">
+    <row r="25" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="17">
         <v>3</v>
       </c>
@@ -2440,7 +2437,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:18" s="18" customFormat="1">
+    <row r="26" spans="1:18" s="18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A26" s="24">
         <v>4</v>
       </c>
@@ -2466,7 +2463,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:18" s="1" customFormat="1">
+    <row r="27" spans="1:18" s="1" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A27" s="25">
         <v>4</v>
       </c>
@@ -2483,7 +2480,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:18">
+    <row r="28" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A28" s="25">
         <v>4</v>
       </c>
@@ -2509,7 +2506,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="29" spans="1:18" s="23" customFormat="1">
+    <row r="29" spans="1:18" s="23" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A29" s="26">
         <v>4</v>
       </c>
@@ -2535,7 +2532,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:18" s="12" customFormat="1">
+    <row r="30" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A30" s="17">
         <v>5</v>
       </c>
@@ -2564,7 +2561,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="31" spans="1:18" s="12" customFormat="1">
+    <row r="31" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="27">
         <v>5</v>
       </c>
@@ -2593,7 +2590,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:18" s="12" customFormat="1">
+    <row r="32" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A32" s="27">
         <v>5</v>
       </c>
@@ -2622,7 +2619,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="33" spans="1:18" s="12" customFormat="1">
+    <row r="33" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A33" s="27">
         <v>5</v>
       </c>
@@ -2651,7 +2648,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="34" spans="1:18" s="12" customFormat="1">
+    <row r="34" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A34" s="12">
         <v>5</v>
       </c>
@@ -2674,7 +2671,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:18" s="12" customFormat="1">
+    <row r="35" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A35" s="12">
         <v>5</v>
       </c>
@@ -2697,7 +2694,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="36" spans="1:18" s="12" customFormat="1">
+    <row r="36" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A36" s="14">
         <v>5</v>
       </c>
@@ -2720,7 +2717,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:18" s="5" customFormat="1">
+    <row r="37" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A37" s="14">
         <v>5</v>
       </c>
@@ -2743,7 +2740,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:18" s="12" customFormat="1">
+    <row r="38" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A38" s="14">
         <v>5</v>
       </c>
@@ -2766,7 +2763,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="39" spans="1:18" s="12" customFormat="1">
+    <row r="39" spans="1:18" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A39" s="14">
         <v>5</v>
       </c>
@@ -2789,7 +2786,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:18">
+    <row r="40" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A40" s="17">
         <v>5</v>
       </c>
@@ -2815,7 +2812,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:18">
+    <row r="41" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A41" s="17">
         <v>5</v>
       </c>
@@ -2838,7 +2835,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:18">
+    <row r="42" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A42" s="17">
         <v>5</v>
       </c>
@@ -2864,7 +2861,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:18" s="5" customFormat="1">
+    <row r="43" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A43" s="17">
         <v>5</v>
       </c>
@@ -2887,7 +2884,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:18" s="5" customFormat="1">
+    <row r="44" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A44" s="17">
         <v>5</v>
       </c>
@@ -2910,7 +2907,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:18" s="5" customFormat="1">
+    <row r="45" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A45" s="17">
         <v>5</v>
       </c>
@@ -2930,7 +2927,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="1:18">
+    <row r="46" spans="1:18" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A46" s="17">
         <v>5</v>
       </c>
@@ -2953,7 +2950,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="47" spans="1:18" s="5" customFormat="1">
+    <row r="47" spans="1:18" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A47" s="17">
         <v>5</v>
       </c>
@@ -2973,7 +2970,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="48" spans="1:18" s="18" customFormat="1">
+    <row r="48" spans="1:18" s="18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A48" s="24">
         <v>6</v>
       </c>
@@ -3002,7 +2999,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:44" s="12" customFormat="1">
+    <row r="49" spans="1:44" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A49" s="25">
         <v>6</v>
       </c>
@@ -3043,7 +3040,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="50" spans="1:44" s="5" customFormat="1">
+    <row r="50" spans="1:44" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A50" s="25">
         <v>6</v>
       </c>
@@ -3063,7 +3060,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="51" spans="1:44" s="5" customFormat="1">
+    <row r="51" spans="1:44" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A51" s="25">
         <v>6</v>
       </c>
@@ -3086,7 +3083,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="52" spans="1:44" s="21" customFormat="1">
+    <row r="52" spans="1:44" s="21" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A52" s="26">
         <v>6</v>
       </c>
@@ -3112,7 +3109,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:44" s="5" customFormat="1">
+    <row r="53" spans="1:44" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
         <v>6</v>
       </c>
@@ -3129,7 +3126,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:44">
+    <row r="54" spans="1:44" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A54" s="17">
         <v>7</v>
       </c>
@@ -3152,7 +3149,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="55" spans="1:44">
+    <row r="55" spans="1:44" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A55" s="17">
         <v>7</v>
       </c>
@@ -3178,7 +3175,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:44">
+    <row r="56" spans="1:44" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A56" s="17">
         <v>7</v>
       </c>
@@ -3204,7 +3201,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:44" s="18" customFormat="1">
+    <row r="57" spans="1:44" s="18" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A57" s="24">
         <v>8</v>
       </c>
@@ -3231,7 +3228,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="58" spans="1:44" s="12" customFormat="1">
+    <row r="58" spans="1:44" s="12" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A58" s="25">
         <v>8</v>
       </c>
@@ -3254,7 +3251,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="1:44" s="21" customFormat="1">
+    <row r="59" spans="1:44" s="21" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A59" s="26">
         <v>8</v>
       </c>
@@ -3314,7 +3311,7 @@
       <c r="AQ59" s="22"/>
       <c r="AR59" s="22"/>
     </row>
-    <row r="60" spans="1:44">
+    <row r="60" spans="1:44" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A60" s="17">
         <v>9</v>
       </c>
@@ -3340,7 +3337,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:44" s="1" customFormat="1">
+    <row r="61" spans="1:44" s="1" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A61" s="30">
         <v>9</v>
       </c>
@@ -3360,13 +3357,13 @@
         <v>185</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="K61" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="62" spans="1:44" s="1" customFormat="1">
+    <row r="62" spans="1:44" s="1" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A62" s="30">
         <v>9</v>
       </c>
@@ -3386,154 +3383,154 @@
         <v>189</v>
       </c>
       <c r="G62" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q62" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="Q62" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="63" spans="1:44" s="29" customFormat="1">
+    </row>
+    <row r="63" spans="1:44" s="29" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A63" s="24">
         <v>10</v>
       </c>
       <c r="B63" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="D63" s="29" t="s">
         <v>192</v>
-      </c>
-      <c r="D63" s="29" t="s">
-        <v>193</v>
       </c>
       <c r="G63" s="29" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="64" spans="1:44" s="5" customFormat="1">
+    <row r="64" spans="1:44" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A64" s="25">
         <v>10</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G64" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:10" s="5" customFormat="1">
+    <row r="65" spans="1:10" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A65" s="25">
         <v>10</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G65" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="5" customFormat="1">
+    <row r="66" spans="1:10" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A66" s="25">
         <v>10</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G66" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="67" spans="1:10" s="22" customFormat="1">
+    <row r="67" spans="1:10" s="22" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A67" s="26">
         <v>10</v>
       </c>
       <c r="B67" s="22" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D67" s="22" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G67" s="22" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="68" spans="1:10"/>
-    <row r="70" spans="1:10">
+    <row r="68" spans="1:10" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="70" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
+        <v>197</v>
+      </c>
+      <c r="G70" t="s">
         <v>198</v>
       </c>
-      <c r="G70" t="s">
+    </row>
+    <row r="71" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B71" t="s">
         <v>199</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10">
-      <c r="B71" t="s">
-        <v>200</v>
       </c>
       <c r="G71" s="1"/>
       <c r="I71" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B72" t="s">
         <v>201</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10">
-      <c r="B72" t="s">
-        <v>202</v>
       </c>
       <c r="G72" s="3"/>
       <c r="I72" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B73" t="s">
         <v>203</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10">
-      <c r="B73" t="s">
-        <v>204</v>
       </c>
       <c r="G73" s="31"/>
       <c r="I73" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="J73" s="32"/>
+    </row>
+    <row r="74" spans="1:10" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B74" t="s">
         <v>205</v>
-      </c>
-      <c r="J73" s="32"/>
-    </row>
-    <row r="74" spans="1:10" ht="14.45" customHeight="1">
-      <c r="B74" t="s">
-        <v>206</v>
       </c>
       <c r="G74" s="33"/>
       <c r="I74" s="32" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J74" s="32"/>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="G75" s="34"/>
       <c r="I75" s="32" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J75" s="32"/>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="G76" s="6"/>
       <c r="I76" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="88" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="89" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="90" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="91" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="92" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="93" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="94" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="95" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="100" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="101" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="102" ht="14.5" x14ac:dyDescent="0.35"/>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R67">
     <sortCondition ref="A2:A67"/>
@@ -3545,145 +3542,145 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H97"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" t="s">
         <v>210</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>211</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>212</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>213</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>214</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>215</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>216</v>
       </c>
-      <c r="H1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>151</v>
       </c>
       <c r="B2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C2" t="s">
         <v>218</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>219</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>220</v>
-      </c>
-      <c r="E2" t="s">
-        <v>221</v>
       </c>
       <c r="F2">
         <v>21</v>
       </c>
       <c r="G2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H2" t="s">
         <v>222</v>
       </c>
-      <c r="H2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>151</v>
       </c>
       <c r="B3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" t="s">
         <v>218</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>219</v>
       </c>
-      <c r="D3" t="s">
-        <v>220</v>
-      </c>
       <c r="E3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F3">
         <v>12</v>
       </c>
       <c r="G3" t="s">
+        <v>221</v>
+      </c>
+      <c r="H3" t="s">
         <v>222</v>
       </c>
-      <c r="H3" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>151</v>
       </c>
       <c r="B4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C4" t="s">
         <v>218</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>219</v>
       </c>
-      <c r="D4" t="s">
-        <v>220</v>
-      </c>
       <c r="E4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F4">
         <v>9</v>
       </c>
       <c r="G4" t="s">
+        <v>221</v>
+      </c>
+      <c r="H4" t="s">
         <v>222</v>
       </c>
-      <c r="H4" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
       </c>
       <c r="D5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" t="s">
         <v>226</v>
       </c>
-      <c r="E5" t="s">
-        <v>226</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>227</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>228</v>
       </c>
-      <c r="H5" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>151</v>
       </c>
@@ -3691,25 +3688,25 @@
         <v>152</v>
       </c>
       <c r="C6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
+        <v>230</v>
+      </c>
+      <c r="H6" t="s">
         <v>231</v>
       </c>
-      <c r="H6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -3717,25 +3714,25 @@
         <v>152</v>
       </c>
       <c r="C7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" t="s">
+        <v>225</v>
+      </c>
+      <c r="E7" t="s">
+        <v>225</v>
+      </c>
+      <c r="F7" t="s">
         <v>233</v>
       </c>
-      <c r="D7" t="s">
-        <v>226</v>
-      </c>
-      <c r="E7" t="s">
-        <v>226</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H7" t="s">
         <v>234</v>
       </c>
-      <c r="G7" t="s">
-        <v>228</v>
-      </c>
-      <c r="H7" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>151</v>
       </c>
@@ -3743,103 +3740,103 @@
         <v>152</v>
       </c>
       <c r="C8" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" t="s">
+        <v>225</v>
+      </c>
+      <c r="F8" t="s">
         <v>236</v>
       </c>
-      <c r="D8" t="s">
-        <v>226</v>
-      </c>
-      <c r="E8" t="s">
-        <v>226</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>227</v>
+      </c>
+      <c r="H8" t="s">
         <v>237</v>
       </c>
-      <c r="G8" t="s">
-        <v>228</v>
-      </c>
-      <c r="H8" t="s">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>238</v>
+      </c>
+      <c r="C9" t="s">
         <v>239</v>
       </c>
-      <c r="B9" t="s">
-        <v>239</v>
-      </c>
-      <c r="C9" t="s">
-        <v>240</v>
-      </c>
       <c r="D9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F9">
         <v>400</v>
       </c>
       <c r="G9" t="s">
+        <v>240</v>
+      </c>
+      <c r="H9" t="s">
         <v>241</v>
       </c>
-      <c r="H9" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F10" t="s">
+        <v>242</v>
+      </c>
+      <c r="G10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H10" t="s">
         <v>243</v>
       </c>
-      <c r="G10" t="s">
-        <v>228</v>
-      </c>
-      <c r="H10" t="s">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B11" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>239</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>245</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>225</v>
+      </c>
+      <c r="E11" t="s">
+        <v>225</v>
+      </c>
+      <c r="F11" t="s">
         <v>246</v>
       </c>
-      <c r="D11" t="s">
-        <v>226</v>
-      </c>
-      <c r="E11" t="s">
-        <v>226</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>227</v>
+      </c>
+      <c r="H11" t="s">
         <v>247</v>
       </c>
-      <c r="G11" t="s">
-        <v>228</v>
-      </c>
-      <c r="H11" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -3847,25 +3844,25 @@
         <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F12">
         <v>104.04</v>
       </c>
       <c r="G12" t="s">
+        <v>249</v>
+      </c>
+      <c r="H12" t="s">
         <v>250</v>
       </c>
-      <c r="H12" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -3873,25 +3870,25 @@
         <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F13">
         <v>51.84</v>
       </c>
       <c r="G13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H13" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -3899,195 +3896,195 @@
         <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F14">
         <v>2000</v>
       </c>
       <c r="G14" t="s">
+        <v>252</v>
+      </c>
+      <c r="H14" t="s">
         <v>253</v>
       </c>
-      <c r="H14" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
       <c r="B15" t="s">
+        <v>254</v>
+      </c>
+      <c r="C15" t="s">
         <v>255</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>225</v>
+      </c>
+      <c r="E15" t="s">
+        <v>225</v>
+      </c>
+      <c r="F15" t="s">
         <v>256</v>
       </c>
-      <c r="D15" t="s">
-        <v>226</v>
-      </c>
-      <c r="E15" t="s">
-        <v>226</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
+        <v>227</v>
+      </c>
+      <c r="H15" t="s">
         <v>257</v>
       </c>
-      <c r="G15" t="s">
-        <v>228</v>
-      </c>
-      <c r="H15" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
+        <v>258</v>
+      </c>
+      <c r="C16" t="s">
+        <v>255</v>
+      </c>
+      <c r="D16" t="s">
+        <v>225</v>
+      </c>
+      <c r="E16" t="s">
+        <v>225</v>
+      </c>
+      <c r="F16" t="s">
         <v>259</v>
       </c>
-      <c r="C16" t="s">
-        <v>256</v>
-      </c>
-      <c r="D16" t="s">
-        <v>226</v>
-      </c>
-      <c r="E16" t="s">
-        <v>226</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>227</v>
+      </c>
+      <c r="H16" t="s">
         <v>260</v>
       </c>
-      <c r="G16" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" t="s">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>262</v>
-      </c>
-      <c r="B17" t="s">
-        <v>263</v>
       </c>
       <c r="C17" t="s">
         <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F17" t="s">
+        <v>263</v>
+      </c>
+      <c r="G17" t="s">
+        <v>227</v>
+      </c>
+      <c r="H17" t="s">
         <v>264</v>
       </c>
-      <c r="G17" t="s">
-        <v>228</v>
-      </c>
-      <c r="H17" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
+      <c r="D18" t="s">
+        <v>219</v>
+      </c>
+      <c r="E18" t="s">
+        <v>266</v>
+      </c>
+      <c r="F18" t="s">
+        <v>267</v>
+      </c>
+      <c r="G18" t="s">
+        <v>268</v>
+      </c>
+      <c r="H18" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>261</v>
+      </c>
+      <c r="B19" t="s">
         <v>262</v>
       </c>
-      <c r="B18" t="s">
-        <v>263</v>
-      </c>
-      <c r="C18" t="s">
-        <v>266</v>
-      </c>
-      <c r="D18" t="s">
-        <v>220</v>
-      </c>
-      <c r="E18" t="s">
-        <v>267</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="C19" t="s">
+        <v>265</v>
+      </c>
+      <c r="D19" t="s">
+        <v>219</v>
+      </c>
+      <c r="E19" t="s">
+        <v>270</v>
+      </c>
+      <c r="F19" t="s">
+        <v>271</v>
+      </c>
+      <c r="G19" t="s">
         <v>268</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H19" t="s">
         <v>269</v>
       </c>
-      <c r="H18" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>261</v>
+      </c>
+      <c r="B20" t="s">
         <v>262</v>
       </c>
-      <c r="B19" t="s">
-        <v>263</v>
-      </c>
-      <c r="C19" t="s">
-        <v>266</v>
-      </c>
-      <c r="D19" t="s">
-        <v>220</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="C20" t="s">
+        <v>265</v>
+      </c>
+      <c r="D20" t="s">
+        <v>219</v>
+      </c>
+      <c r="E20" t="s">
+        <v>272</v>
+      </c>
+      <c r="F20" t="s">
         <v>271</v>
       </c>
-      <c r="F19" t="s">
-        <v>272</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="G20" t="s">
+        <v>268</v>
+      </c>
+      <c r="H20" t="s">
         <v>269</v>
       </c>
-      <c r="H19" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" t="s">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>261</v>
+      </c>
+      <c r="B21" t="s">
         <v>262</v>
       </c>
-      <c r="B20" t="s">
-        <v>263</v>
-      </c>
-      <c r="C20" t="s">
-        <v>266</v>
-      </c>
-      <c r="D20" t="s">
-        <v>220</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="C21" t="s">
         <v>273</v>
       </c>
-      <c r="F20" t="s">
-        <v>272</v>
-      </c>
-      <c r="G20" t="s">
-        <v>269</v>
-      </c>
-      <c r="H20" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>262</v>
-      </c>
-      <c r="B21" t="s">
-        <v>263</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>274</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>275</v>
-      </c>
-      <c r="E21" t="s">
-        <v>276</v>
       </c>
       <c r="F21">
         <v>100</v>
@@ -4096,24 +4093,24 @@
         <v>105</v>
       </c>
       <c r="H21" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>261</v>
+      </c>
+      <c r="B22" t="s">
+        <v>262</v>
+      </c>
+      <c r="C22" t="s">
+        <v>273</v>
+      </c>
+      <c r="D22" t="s">
+        <v>274</v>
+      </c>
+      <c r="E22" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>262</v>
-      </c>
-      <c r="B22" t="s">
-        <v>263</v>
-      </c>
-      <c r="C22" t="s">
-        <v>274</v>
-      </c>
-      <c r="D22" t="s">
-        <v>275</v>
-      </c>
-      <c r="E22" t="s">
-        <v>278</v>
       </c>
       <c r="F22">
         <v>300</v>
@@ -4122,24 +4119,24 @@
         <v>105</v>
       </c>
       <c r="H22" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>261</v>
+      </c>
+      <c r="B23" t="s">
         <v>262</v>
       </c>
-      <c r="B23" t="s">
-        <v>263</v>
-      </c>
       <c r="C23" t="s">
+        <v>273</v>
+      </c>
+      <c r="D23" t="s">
         <v>274</v>
       </c>
-      <c r="D23" t="s">
-        <v>275</v>
-      </c>
       <c r="E23" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F23">
         <v>450</v>
@@ -4148,24 +4145,24 @@
         <v>105</v>
       </c>
       <c r="H23" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>261</v>
+      </c>
+      <c r="B24" t="s">
         <v>262</v>
       </c>
-      <c r="B24" t="s">
-        <v>263</v>
-      </c>
       <c r="C24" t="s">
+        <v>273</v>
+      </c>
+      <c r="D24" t="s">
         <v>274</v>
       </c>
-      <c r="D24" t="s">
-        <v>275</v>
-      </c>
       <c r="E24" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F24">
         <v>675</v>
@@ -4174,24 +4171,24 @@
         <v>105</v>
       </c>
       <c r="H24" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>261</v>
+      </c>
+      <c r="B25" t="s">
         <v>262</v>
       </c>
-      <c r="B25" t="s">
-        <v>263</v>
-      </c>
       <c r="C25" t="s">
+        <v>273</v>
+      </c>
+      <c r="D25" t="s">
         <v>274</v>
       </c>
-      <c r="D25" t="s">
-        <v>275</v>
-      </c>
       <c r="E25" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F25">
         <v>100</v>
@@ -4200,24 +4197,24 @@
         <v>105</v>
       </c>
       <c r="H25" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>261</v>
+      </c>
+      <c r="B26" t="s">
         <v>262</v>
       </c>
-      <c r="B26" t="s">
-        <v>263</v>
-      </c>
       <c r="C26" t="s">
+        <v>273</v>
+      </c>
+      <c r="D26" t="s">
         <v>274</v>
       </c>
-      <c r="D26" t="s">
-        <v>275</v>
-      </c>
       <c r="E26" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F26">
         <v>300</v>
@@ -4226,24 +4223,24 @@
         <v>105</v>
       </c>
       <c r="H26" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>261</v>
+      </c>
+      <c r="B27" t="s">
         <v>262</v>
       </c>
-      <c r="B27" t="s">
-        <v>263</v>
-      </c>
       <c r="C27" t="s">
+        <v>273</v>
+      </c>
+      <c r="D27" t="s">
         <v>274</v>
       </c>
-      <c r="D27" t="s">
-        <v>275</v>
-      </c>
       <c r="E27" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F27">
         <v>450</v>
@@ -4252,24 +4249,24 @@
         <v>105</v>
       </c>
       <c r="H27" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>261</v>
+      </c>
+      <c r="B28" t="s">
         <v>262</v>
       </c>
-      <c r="B28" t="s">
-        <v>263</v>
-      </c>
       <c r="C28" t="s">
+        <v>273</v>
+      </c>
+      <c r="D28" t="s">
         <v>274</v>
       </c>
-      <c r="D28" t="s">
-        <v>275</v>
-      </c>
       <c r="E28" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F28">
         <v>675</v>
@@ -4278,24 +4275,24 @@
         <v>105</v>
       </c>
       <c r="H28" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
+        <v>261</v>
+      </c>
+      <c r="B29" t="s">
         <v>262</v>
       </c>
-      <c r="B29" t="s">
-        <v>263</v>
-      </c>
       <c r="C29" t="s">
+        <v>273</v>
+      </c>
+      <c r="D29" t="s">
         <v>274</v>
       </c>
-      <c r="D29" t="s">
-        <v>275</v>
-      </c>
       <c r="E29" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F29">
         <v>150</v>
@@ -4304,24 +4301,24 @@
         <v>105</v>
       </c>
       <c r="H29" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>261</v>
+      </c>
+      <c r="B30" t="s">
         <v>262</v>
       </c>
-      <c r="B30" t="s">
-        <v>263</v>
-      </c>
       <c r="C30" t="s">
+        <v>273</v>
+      </c>
+      <c r="D30" t="s">
         <v>274</v>
       </c>
-      <c r="D30" t="s">
-        <v>275</v>
-      </c>
       <c r="E30" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F30">
         <v>200</v>
@@ -4330,24 +4327,24 @@
         <v>105</v>
       </c>
       <c r="H30" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
+        <v>261</v>
+      </c>
+      <c r="B31" t="s">
         <v>262</v>
       </c>
-      <c r="B31" t="s">
-        <v>263</v>
-      </c>
       <c r="C31" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" t="s">
         <v>274</v>
       </c>
-      <c r="D31" t="s">
-        <v>275</v>
-      </c>
       <c r="E31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F31">
         <v>300</v>
@@ -4356,24 +4353,24 @@
         <v>105</v>
       </c>
       <c r="H31" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>261</v>
+      </c>
+      <c r="B32" t="s">
         <v>262</v>
       </c>
-      <c r="B32" t="s">
-        <v>263</v>
-      </c>
       <c r="C32" t="s">
+        <v>273</v>
+      </c>
+      <c r="D32" t="s">
         <v>274</v>
       </c>
-      <c r="D32" t="s">
-        <v>275</v>
-      </c>
       <c r="E32" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F32">
         <v>450</v>
@@ -4382,24 +4379,24 @@
         <v>105</v>
       </c>
       <c r="H32" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>261</v>
+      </c>
+      <c r="B33" t="s">
         <v>262</v>
       </c>
-      <c r="B33" t="s">
-        <v>263</v>
-      </c>
       <c r="C33" t="s">
+        <v>273</v>
+      </c>
+      <c r="D33" t="s">
         <v>274</v>
       </c>
-      <c r="D33" t="s">
-        <v>275</v>
-      </c>
       <c r="E33" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F33">
         <v>675</v>
@@ -4408,24 +4405,24 @@
         <v>105</v>
       </c>
       <c r="H33" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>261</v>
+      </c>
+      <c r="B34" t="s">
         <v>262</v>
       </c>
-      <c r="B34" t="s">
-        <v>263</v>
-      </c>
       <c r="C34" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D34" t="s">
+        <v>274</v>
+      </c>
+      <c r="E34" t="s">
         <v>275</v>
-      </c>
-      <c r="E34" t="s">
-        <v>276</v>
       </c>
       <c r="F34">
         <v>150</v>
@@ -4434,24 +4431,24 @@
         <v>105</v>
       </c>
       <c r="H34" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>261</v>
+      </c>
+      <c r="B35" t="s">
+        <v>262</v>
+      </c>
+      <c r="C35" t="s">
+        <v>289</v>
+      </c>
+      <c r="D35" t="s">
+        <v>274</v>
+      </c>
+      <c r="E35" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" t="s">
-        <v>262</v>
-      </c>
-      <c r="B35" t="s">
-        <v>263</v>
-      </c>
-      <c r="C35" t="s">
-        <v>290</v>
-      </c>
-      <c r="D35" t="s">
-        <v>275</v>
-      </c>
-      <c r="E35" t="s">
-        <v>278</v>
       </c>
       <c r="F35">
         <v>450</v>
@@ -4460,24 +4457,24 @@
         <v>105</v>
       </c>
       <c r="H35" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>261</v>
+      </c>
+      <c r="B36" t="s">
         <v>262</v>
       </c>
-      <c r="B36" t="s">
-        <v>263</v>
-      </c>
       <c r="C36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D36" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E36" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F36">
         <v>675</v>
@@ -4486,24 +4483,24 @@
         <v>105</v>
       </c>
       <c r="H36" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>261</v>
+      </c>
+      <c r="B37" t="s">
         <v>262</v>
       </c>
-      <c r="B37" t="s">
-        <v>263</v>
-      </c>
       <c r="C37" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D37" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E37" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F37">
         <v>1000</v>
@@ -4512,24 +4509,24 @@
         <v>105</v>
       </c>
       <c r="H37" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>261</v>
+      </c>
+      <c r="B38" t="s">
         <v>262</v>
       </c>
-      <c r="B38" t="s">
-        <v>263</v>
-      </c>
       <c r="C38" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D38" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E38" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F38">
         <v>150</v>
@@ -4538,24 +4535,24 @@
         <v>105</v>
       </c>
       <c r="H38" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>261</v>
+      </c>
+      <c r="B39" t="s">
         <v>262</v>
       </c>
-      <c r="B39" t="s">
-        <v>263</v>
-      </c>
       <c r="C39" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D39" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E39" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F39">
         <v>450</v>
@@ -4564,24 +4561,24 @@
         <v>105</v>
       </c>
       <c r="H39" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
+        <v>261</v>
+      </c>
+      <c r="B40" t="s">
         <v>262</v>
       </c>
-      <c r="B40" t="s">
-        <v>263</v>
-      </c>
       <c r="C40" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D40" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E40" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F40">
         <v>675</v>
@@ -4590,24 +4587,24 @@
         <v>105</v>
       </c>
       <c r="H40" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>261</v>
+      </c>
+      <c r="B41" t="s">
         <v>262</v>
       </c>
-      <c r="B41" t="s">
-        <v>263</v>
-      </c>
       <c r="C41" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D41" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E41" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F41">
         <v>1000</v>
@@ -4616,24 +4613,24 @@
         <v>105</v>
       </c>
       <c r="H41" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
+        <v>261</v>
+      </c>
+      <c r="B42" t="s">
         <v>262</v>
       </c>
-      <c r="B42" t="s">
-        <v>263</v>
-      </c>
       <c r="C42" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D42" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E42" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F42">
         <v>225</v>
@@ -4642,24 +4639,24 @@
         <v>105</v>
       </c>
       <c r="H42" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
+        <v>261</v>
+      </c>
+      <c r="B43" t="s">
         <v>262</v>
       </c>
-      <c r="B43" t="s">
-        <v>263</v>
-      </c>
       <c r="C43" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D43" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E43" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F43">
         <v>300</v>
@@ -4668,24 +4665,24 @@
         <v>105</v>
       </c>
       <c r="H43" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
+        <v>261</v>
+      </c>
+      <c r="B44" t="s">
         <v>262</v>
       </c>
-      <c r="B44" t="s">
-        <v>263</v>
-      </c>
       <c r="C44" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D44" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E44" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F44">
         <v>450</v>
@@ -4694,24 +4691,24 @@
         <v>105</v>
       </c>
       <c r="H44" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
+        <v>261</v>
+      </c>
+      <c r="B45" t="s">
         <v>262</v>
       </c>
-      <c r="B45" t="s">
-        <v>263</v>
-      </c>
       <c r="C45" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D45" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E45" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F45">
         <v>675</v>
@@ -4720,24 +4717,24 @@
         <v>105</v>
       </c>
       <c r="H45" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
+        <v>261</v>
+      </c>
+      <c r="B46" t="s">
         <v>262</v>
       </c>
-      <c r="B46" t="s">
-        <v>263</v>
-      </c>
       <c r="C46" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D46" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F46">
         <v>1000</v>
@@ -4746,102 +4743,102 @@
         <v>105</v>
       </c>
       <c r="H46" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
+        <v>261</v>
+      </c>
+      <c r="B47" t="s">
         <v>262</v>
       </c>
-      <c r="B47" t="s">
-        <v>263</v>
-      </c>
       <c r="C47" t="s">
+        <v>290</v>
+      </c>
+      <c r="D47" t="s">
+        <v>219</v>
+      </c>
+      <c r="E47" t="s">
+        <v>266</v>
+      </c>
+      <c r="F47" t="s">
         <v>291</v>
       </c>
-      <c r="D47" t="s">
-        <v>220</v>
-      </c>
-      <c r="E47" t="s">
-        <v>267</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
+        <v>268</v>
+      </c>
+      <c r="H47" t="s">
         <v>292</v>
       </c>
-      <c r="G47" t="s">
-        <v>269</v>
-      </c>
-      <c r="H47" t="s">
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>261</v>
+      </c>
+      <c r="B48" t="s">
+        <v>262</v>
+      </c>
+      <c r="C48" t="s">
+        <v>290</v>
+      </c>
+      <c r="D48" t="s">
+        <v>219</v>
+      </c>
+      <c r="E48" t="s">
+        <v>270</v>
+      </c>
+      <c r="F48" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" t="s">
+      <c r="G48" t="s">
+        <v>268</v>
+      </c>
+      <c r="H48" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>261</v>
+      </c>
+      <c r="B49" t="s">
         <v>262</v>
       </c>
-      <c r="B48" t="s">
-        <v>263</v>
-      </c>
-      <c r="C48" t="s">
-        <v>291</v>
-      </c>
-      <c r="D48" t="s">
-        <v>220</v>
-      </c>
-      <c r="E48" t="s">
-        <v>271</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="C49" t="s">
+        <v>290</v>
+      </c>
+      <c r="D49" t="s">
+        <v>219</v>
+      </c>
+      <c r="E49" t="s">
+        <v>272</v>
+      </c>
+      <c r="F49" t="s">
         <v>294</v>
       </c>
-      <c r="G48" t="s">
-        <v>269</v>
-      </c>
-      <c r="H48" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" t="s">
+      <c r="G49" t="s">
+        <v>268</v>
+      </c>
+      <c r="H49" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>261</v>
+      </c>
+      <c r="B50" t="s">
         <v>262</v>
       </c>
-      <c r="B49" t="s">
-        <v>263</v>
-      </c>
-      <c r="C49" t="s">
-        <v>291</v>
-      </c>
-      <c r="D49" t="s">
-        <v>220</v>
-      </c>
-      <c r="E49" t="s">
-        <v>273</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="C50" t="s">
         <v>295</v>
       </c>
-      <c r="G49" t="s">
-        <v>269</v>
-      </c>
-      <c r="H49" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
-      <c r="A50" t="s">
-        <v>262</v>
-      </c>
-      <c r="B50" t="s">
-        <v>263</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
+        <v>274</v>
+      </c>
+      <c r="E50" t="s">
         <v>296</v>
-      </c>
-      <c r="D50" t="s">
-        <v>275</v>
-      </c>
-      <c r="E50" t="s">
-        <v>297</v>
       </c>
       <c r="F50">
         <v>15</v>
@@ -4850,24 +4847,24 @@
         <v>105</v>
       </c>
       <c r="H50" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>261</v>
+      </c>
+      <c r="B51" t="s">
+        <v>262</v>
+      </c>
+      <c r="C51" t="s">
+        <v>295</v>
+      </c>
+      <c r="D51" t="s">
+        <v>274</v>
+      </c>
+      <c r="E51" t="s">
         <v>298</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51" t="s">
-        <v>262</v>
-      </c>
-      <c r="B51" t="s">
-        <v>263</v>
-      </c>
-      <c r="C51" t="s">
-        <v>296</v>
-      </c>
-      <c r="D51" t="s">
-        <v>275</v>
-      </c>
-      <c r="E51" t="s">
-        <v>299</v>
       </c>
       <c r="F51">
         <v>45</v>
@@ -4876,24 +4873,24 @@
         <v>105</v>
       </c>
       <c r="H51" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
+        <v>261</v>
+      </c>
+      <c r="B52" t="s">
         <v>262</v>
       </c>
-      <c r="B52" t="s">
-        <v>263</v>
-      </c>
       <c r="C52" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D52" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E52" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F52">
         <v>80</v>
@@ -4902,24 +4899,24 @@
         <v>105</v>
       </c>
       <c r="H52" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
+        <v>261</v>
+      </c>
+      <c r="B53" t="s">
         <v>262</v>
       </c>
-      <c r="B53" t="s">
-        <v>263</v>
-      </c>
       <c r="C53" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D53" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E53" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F53">
         <v>80</v>
@@ -4928,24 +4925,24 @@
         <v>105</v>
       </c>
       <c r="H53" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>261</v>
+      </c>
+      <c r="B54" t="s">
         <v>262</v>
       </c>
-      <c r="B54" t="s">
-        <v>263</v>
-      </c>
       <c r="C54" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D54" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E54" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F54">
         <v>115</v>
@@ -4954,24 +4951,24 @@
         <v>105</v>
       </c>
       <c r="H54" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
+        <v>261</v>
+      </c>
+      <c r="B55" t="s">
         <v>262</v>
       </c>
-      <c r="B55" t="s">
-        <v>263</v>
-      </c>
       <c r="C55" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D55" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E55" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F55">
         <v>150</v>
@@ -4980,24 +4977,24 @@
         <v>105</v>
       </c>
       <c r="H55" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
+        <v>261</v>
+      </c>
+      <c r="B56" t="s">
         <v>262</v>
       </c>
-      <c r="B56" t="s">
-        <v>263</v>
-      </c>
       <c r="C56" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D56" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E56" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F56">
         <v>150</v>
@@ -5006,24 +5003,24 @@
         <v>105</v>
       </c>
       <c r="H56" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
+        <v>261</v>
+      </c>
+      <c r="B57" t="s">
         <v>262</v>
       </c>
-      <c r="B57" t="s">
-        <v>263</v>
-      </c>
       <c r="C57" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D57" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E57" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F57">
         <v>225</v>
@@ -5032,24 +5029,24 @@
         <v>105</v>
       </c>
       <c r="H57" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
+        <v>261</v>
+      </c>
+      <c r="B58" t="s">
         <v>262</v>
       </c>
-      <c r="B58" t="s">
-        <v>263</v>
-      </c>
       <c r="C58" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D58" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E58" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F58">
         <v>300</v>
@@ -5058,24 +5055,24 @@
         <v>105</v>
       </c>
       <c r="H58" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
+        <v>261</v>
+      </c>
+      <c r="B59" t="s">
         <v>262</v>
       </c>
-      <c r="B59" t="s">
-        <v>263</v>
-      </c>
       <c r="C59" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D59" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E59" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F59">
         <v>80</v>
@@ -5084,24 +5081,24 @@
         <v>105</v>
       </c>
       <c r="H59" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
+        <v>261</v>
+      </c>
+      <c r="B60" t="s">
         <v>262</v>
       </c>
-      <c r="B60" t="s">
-        <v>263</v>
-      </c>
       <c r="C60" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D60" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E60" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F60">
         <v>115</v>
@@ -5110,24 +5107,24 @@
         <v>105</v>
       </c>
       <c r="H60" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
+        <v>261</v>
+      </c>
+      <c r="B61" t="s">
         <v>262</v>
       </c>
-      <c r="B61" t="s">
-        <v>263</v>
-      </c>
       <c r="C61" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D61" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E61" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F61">
         <v>150</v>
@@ -5136,24 +5133,24 @@
         <v>105</v>
       </c>
       <c r="H61" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
+        <v>261</v>
+      </c>
+      <c r="B62" t="s">
         <v>262</v>
       </c>
-      <c r="B62" t="s">
-        <v>263</v>
-      </c>
       <c r="C62" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D62" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E62" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F62">
         <v>150</v>
@@ -5162,24 +5159,24 @@
         <v>105</v>
       </c>
       <c r="H62" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
+        <v>261</v>
+      </c>
+      <c r="B63" t="s">
         <v>262</v>
       </c>
-      <c r="B63" t="s">
-        <v>263</v>
-      </c>
       <c r="C63" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D63" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E63" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F63">
         <v>225</v>
@@ -5188,24 +5185,24 @@
         <v>105</v>
       </c>
       <c r="H63" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
+        <v>261</v>
+      </c>
+      <c r="B64" t="s">
         <v>262</v>
       </c>
-      <c r="B64" t="s">
-        <v>263</v>
-      </c>
       <c r="C64" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D64" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E64" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F64">
         <v>300</v>
@@ -5214,24 +5211,24 @@
         <v>105</v>
       </c>
       <c r="H64" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
+        <v>261</v>
+      </c>
+      <c r="B65" t="s">
         <v>262</v>
       </c>
-      <c r="B65" t="s">
-        <v>263</v>
-      </c>
       <c r="C65" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D65" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E65" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F65">
         <v>150</v>
@@ -5240,24 +5237,24 @@
         <v>105</v>
       </c>
       <c r="H65" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
+        <v>261</v>
+      </c>
+      <c r="B66" t="s">
         <v>262</v>
       </c>
-      <c r="B66" t="s">
-        <v>263</v>
-      </c>
       <c r="C66" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D66" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E66" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F66">
         <v>225</v>
@@ -5266,24 +5263,24 @@
         <v>105</v>
       </c>
       <c r="H66" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
+        <v>261</v>
+      </c>
+      <c r="B67" t="s">
         <v>262</v>
       </c>
-      <c r="B67" t="s">
-        <v>263</v>
-      </c>
       <c r="C67" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D67" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E67" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F67">
         <v>300</v>
@@ -5292,712 +5289,712 @@
         <v>105</v>
       </c>
       <c r="H67" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>261</v>
+      </c>
+      <c r="B68" t="s">
+        <v>262</v>
+      </c>
+      <c r="C68" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="68" spans="1:8">
-      <c r="A68" t="s">
-        <v>262</v>
-      </c>
-      <c r="B68" t="s">
-        <v>263</v>
-      </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
+        <v>274</v>
+      </c>
+      <c r="E68" t="s">
+        <v>296</v>
+      </c>
+      <c r="F68" t="s">
         <v>309</v>
-      </c>
-      <c r="D68" t="s">
-        <v>275</v>
-      </c>
-      <c r="E68" t="s">
-        <v>297</v>
-      </c>
-      <c r="F68" t="s">
-        <v>310</v>
       </c>
       <c r="G68" t="s">
         <v>42</v>
       </c>
       <c r="H68" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>261</v>
+      </c>
+      <c r="B69" t="s">
+        <v>262</v>
+      </c>
+      <c r="C69" t="s">
+        <v>308</v>
+      </c>
+      <c r="D69" t="s">
+        <v>274</v>
+      </c>
+      <c r="E69" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="69" spans="1:8">
-      <c r="A69" t="s">
-        <v>262</v>
-      </c>
-      <c r="B69" t="s">
-        <v>263</v>
-      </c>
-      <c r="C69" t="s">
-        <v>309</v>
-      </c>
-      <c r="D69" t="s">
-        <v>275</v>
-      </c>
-      <c r="E69" t="s">
-        <v>299</v>
-      </c>
       <c r="F69" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G69" t="s">
         <v>42</v>
       </c>
       <c r="H69" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
+        <v>261</v>
+      </c>
+      <c r="B70" t="s">
         <v>262</v>
       </c>
-      <c r="B70" t="s">
-        <v>263</v>
-      </c>
       <c r="C70" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D70" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E70" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F70" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G70" t="s">
         <v>42</v>
       </c>
       <c r="H70" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
+        <v>261</v>
+      </c>
+      <c r="B71" t="s">
         <v>262</v>
       </c>
-      <c r="B71" t="s">
-        <v>263</v>
-      </c>
       <c r="C71" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D71" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E71" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F71" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G71" t="s">
         <v>42</v>
       </c>
       <c r="H71" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>261</v>
+      </c>
+      <c r="B72" t="s">
         <v>262</v>
       </c>
-      <c r="B72" t="s">
-        <v>263</v>
-      </c>
       <c r="C72" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D72" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E72" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F72" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G72" t="s">
         <v>42</v>
       </c>
       <c r="H72" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>261</v>
+      </c>
+      <c r="B73" t="s">
         <v>262</v>
       </c>
-      <c r="B73" t="s">
-        <v>263</v>
-      </c>
       <c r="C73" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D73" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E73" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F73" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G73" t="s">
         <v>42</v>
       </c>
       <c r="H73" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
+        <v>261</v>
+      </c>
+      <c r="B74" t="s">
         <v>262</v>
       </c>
-      <c r="B74" t="s">
-        <v>263</v>
-      </c>
       <c r="C74" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D74" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E74" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F74" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G74" t="s">
         <v>42</v>
       </c>
       <c r="H74" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
+        <v>261</v>
+      </c>
+      <c r="B75" t="s">
         <v>262</v>
       </c>
-      <c r="B75" t="s">
-        <v>263</v>
-      </c>
       <c r="C75" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D75" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E75" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F75" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G75" t="s">
         <v>42</v>
       </c>
       <c r="H75" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
+        <v>261</v>
+      </c>
+      <c r="B76" t="s">
         <v>262</v>
       </c>
-      <c r="B76" t="s">
-        <v>263</v>
-      </c>
       <c r="C76" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D76" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E76" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F76" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G76" t="s">
         <v>42</v>
       </c>
       <c r="H76" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
+        <v>318</v>
+      </c>
+      <c r="B77" t="s">
         <v>319</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>320</v>
       </c>
-      <c r="C77" t="s">
-        <v>321</v>
-      </c>
       <c r="D77" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E77" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F77">
         <v>1</v>
       </c>
       <c r="G77" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H77" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>318</v>
+      </c>
+      <c r="B78" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="78" spans="1:8">
-      <c r="A78" t="s">
-        <v>319</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>323</v>
       </c>
-      <c r="C78" t="s">
-        <v>324</v>
-      </c>
       <c r="D78" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E78" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F78">
         <v>1</v>
       </c>
       <c r="G78" t="s">
+        <v>324</v>
+      </c>
+      <c r="H78" t="s">
         <v>325</v>
       </c>
-      <c r="H78" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8">
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B79" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C79" t="s">
         <v>28</v>
       </c>
       <c r="D79" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E79" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F79" t="s">
+        <v>326</v>
+      </c>
+      <c r="G79" t="s">
+        <v>227</v>
+      </c>
+      <c r="H79" t="s">
         <v>327</v>
       </c>
-      <c r="G79" t="s">
-        <v>228</v>
-      </c>
-      <c r="H79" t="s">
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>318</v>
+      </c>
+      <c r="B80" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="80" spans="1:8">
-      <c r="A80" t="s">
-        <v>319</v>
-      </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>329</v>
       </c>
-      <c r="C80" t="s">
-        <v>330</v>
-      </c>
       <c r="D80" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E80" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F80">
         <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H80" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="81" spans="1:8">
-      <c r="A81" t="s">
+      <c r="B81" t="s">
         <v>332</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>333</v>
       </c>
-      <c r="C81" t="s">
-        <v>334</v>
-      </c>
       <c r="D81" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E81" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F81">
         <v>100</v>
       </c>
       <c r="G81" t="s">
+        <v>334</v>
+      </c>
+      <c r="H81" t="s">
         <v>335</v>
       </c>
-      <c r="H81" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8">
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
+        <v>331</v>
+      </c>
+      <c r="B82" t="s">
         <v>332</v>
-      </c>
-      <c r="B82" t="s">
-        <v>333</v>
       </c>
       <c r="C82" t="s">
         <v>28</v>
       </c>
       <c r="D82" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E82" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F82" t="s">
+        <v>336</v>
+      </c>
+      <c r="G82" t="s">
+        <v>227</v>
+      </c>
+      <c r="H82" t="s">
         <v>337</v>
       </c>
-      <c r="G82" t="s">
-        <v>228</v>
-      </c>
-      <c r="H82" t="s">
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>331</v>
+      </c>
+      <c r="B83" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="83" spans="1:8">
-      <c r="A83" t="s">
-        <v>332</v>
-      </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>339</v>
       </c>
-      <c r="C83" t="s">
-        <v>340</v>
-      </c>
       <c r="D83" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E83" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F83">
         <v>1</v>
       </c>
       <c r="G83" t="s">
+        <v>340</v>
+      </c>
+      <c r="H83" t="s">
         <v>341</v>
       </c>
-      <c r="H83" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8">
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B84" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C84" t="s">
         <v>28</v>
       </c>
       <c r="D84" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E84" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F84" t="s">
+        <v>342</v>
+      </c>
+      <c r="G84" t="s">
+        <v>227</v>
+      </c>
+      <c r="H84" t="s">
         <v>343</v>
       </c>
-      <c r="G84" t="s">
-        <v>228</v>
-      </c>
-      <c r="H84" t="s">
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>331</v>
+      </c>
+      <c r="B85" t="s">
+        <v>332</v>
+      </c>
+      <c r="C85" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="85" spans="1:8">
-      <c r="A85" t="s">
-        <v>332</v>
-      </c>
-      <c r="B85" t="s">
-        <v>333</v>
-      </c>
-      <c r="C85" t="s">
-        <v>345</v>
-      </c>
       <c r="D85" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E85" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F85">
         <v>10</v>
       </c>
       <c r="G85" t="s">
+        <v>345</v>
+      </c>
+      <c r="H85" t="s">
         <v>346</v>
       </c>
-      <c r="H85" t="s">
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="86" spans="1:8">
-      <c r="A86" t="s">
+      <c r="B86" t="s">
         <v>348</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
         <v>349</v>
       </c>
-      <c r="C86" t="s">
-        <v>350</v>
-      </c>
       <c r="D86" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E86" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F86">
         <v>1</v>
       </c>
       <c r="G86" t="s">
+        <v>350</v>
+      </c>
+      <c r="H86" t="s">
         <v>351</v>
       </c>
-      <c r="H86" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8">
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
+        <v>347</v>
+      </c>
+      <c r="B87" t="s">
         <v>348</v>
-      </c>
-      <c r="B87" t="s">
-        <v>349</v>
       </c>
       <c r="C87" t="s">
         <v>28</v>
       </c>
       <c r="D87" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E87" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F87" t="s">
+        <v>352</v>
+      </c>
+      <c r="G87" t="s">
+        <v>227</v>
+      </c>
+      <c r="H87" t="s">
         <v>353</v>
       </c>
-      <c r="G87" t="s">
-        <v>228</v>
-      </c>
-      <c r="H87" t="s">
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>347</v>
+      </c>
+      <c r="B88" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="88" spans="1:8">
-      <c r="A88" t="s">
-        <v>348</v>
-      </c>
-      <c r="B88" t="s">
+      <c r="C88" t="s">
         <v>355</v>
       </c>
-      <c r="C88" t="s">
-        <v>356</v>
-      </c>
       <c r="D88" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E88" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F88">
         <v>500</v>
       </c>
       <c r="G88" t="s">
+        <v>356</v>
+      </c>
+      <c r="H88" t="s">
         <v>357</v>
       </c>
-      <c r="H88" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8">
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B89" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C89" t="s">
         <v>28</v>
       </c>
       <c r="D89" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E89" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F89" t="s">
+        <v>358</v>
+      </c>
+      <c r="G89" t="s">
+        <v>227</v>
+      </c>
+      <c r="H89" t="s">
         <v>359</v>
       </c>
-      <c r="G89" t="s">
-        <v>228</v>
-      </c>
-      <c r="H89" t="s">
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="90" spans="1:8">
-      <c r="A90" t="s">
+      <c r="B90" t="s">
         <v>361</v>
       </c>
-      <c r="B90" t="s">
-        <v>362</v>
-      </c>
       <c r="C90" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D90" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E90" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F90">
         <v>250</v>
       </c>
       <c r="G90" t="s">
+        <v>362</v>
+      </c>
+      <c r="H90" t="s">
         <v>363</v>
       </c>
-      <c r="H90" t="s">
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>360</v>
+      </c>
+      <c r="B91" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="91" spans="1:8">
-      <c r="A91" t="s">
-        <v>361</v>
-      </c>
-      <c r="B91" t="s">
-        <v>365</v>
-      </c>
       <c r="C91" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D91" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E91" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F91">
         <v>200</v>
       </c>
       <c r="G91" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H91" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>360</v>
+      </c>
+      <c r="B92" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="92" spans="1:8">
-      <c r="A92" t="s">
-        <v>361</v>
-      </c>
-      <c r="B92" t="s">
-        <v>367</v>
-      </c>
       <c r="C92" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D92" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E92" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F92">
         <v>250</v>
       </c>
       <c r="G92" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H92" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>360</v>
+      </c>
+      <c r="B93" t="s">
         <v>368</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8">
-      <c r="A93" t="s">
-        <v>361</v>
-      </c>
-      <c r="B93" t="s">
-        <v>369</v>
       </c>
       <c r="C93" t="s">
         <v>28</v>
       </c>
       <c r="D93" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E93" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F93" t="s">
+        <v>369</v>
+      </c>
+      <c r="G93" t="s">
+        <v>227</v>
+      </c>
+      <c r="H93" t="s">
         <v>370</v>
       </c>
-      <c r="G93" t="s">
-        <v>228</v>
-      </c>
-      <c r="H93" t="s">
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>360</v>
+      </c>
+      <c r="B94" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="94" spans="1:8">
-      <c r="A94" t="s">
-        <v>361</v>
-      </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
+        <v>255</v>
+      </c>
+      <c r="D94" t="s">
+        <v>225</v>
+      </c>
+      <c r="E94" t="s">
+        <v>225</v>
+      </c>
+      <c r="F94" t="s">
         <v>372</v>
       </c>
-      <c r="C94" t="s">
-        <v>256</v>
-      </c>
-      <c r="D94" t="s">
-        <v>226</v>
-      </c>
-      <c r="E94" t="s">
-        <v>226</v>
-      </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H94" t="s">
         <v>373</v>
       </c>
-      <c r="G94" t="s">
-        <v>228</v>
-      </c>
-      <c r="H94" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8">
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>26</v>
       </c>
@@ -6008,22 +6005,22 @@
         <v>28</v>
       </c>
       <c r="D95" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E95" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F95" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G95" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H95" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="96" spans="1:8">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>26</v>
       </c>
@@ -6034,22 +6031,22 @@
         <v>28</v>
       </c>
       <c r="D96" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E96" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F96" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G96" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H96" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="97" spans="1:8">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>26</v>
       </c>
@@ -6060,19 +6057,19 @@
         <v>28</v>
       </c>
       <c r="D97" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E97" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F97" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G97" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H97" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -6083,14 +6080,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9B6005-6F43-4EB4-8661-C70A2093261E}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -6098,21 +6095,21 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
+        <v>375</v>
+      </c>
+      <c r="D1" t="s">
         <v>376</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>377</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>378</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>379</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>380</v>
       </c>
       <c r="C2">
         <v>30</v>
@@ -6124,9 +6121,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C3">
         <v>60</v>
@@ -6138,9 +6135,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C4">
         <v>90</v>
@@ -6152,9 +6149,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C5">
         <v>120</v>
@@ -6166,9 +6163,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C6">
         <v>180</v>
@@ -6180,9 +6177,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C7">
         <v>240</v>
@@ -6194,9 +6191,9 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C8">
         <v>30</v>
@@ -6208,9 +6205,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C9">
         <v>60</v>
@@ -6222,9 +6219,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C10">
         <v>90</v>
@@ -6236,9 +6233,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C11">
         <v>120</v>
@@ -6250,9 +6247,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C12">
         <v>180</v>
@@ -6264,9 +6261,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C13">
         <v>240</v>
@@ -6278,9 +6275,9 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C14">
         <v>60</v>
@@ -6292,9 +6289,9 @@
         <v>600</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C15">
         <v>90</v>
@@ -6306,9 +6303,9 @@
         <v>600</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C16">
         <v>120</v>
@@ -6320,12 +6317,12 @@
         <v>600</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>382</v>
+      </c>
+      <c r="B17" t="s">
         <v>383</v>
-      </c>
-      <c r="B17" t="s">
-        <v>384</v>
       </c>
       <c r="C17">
         <v>60</v>
@@ -6334,12 +6331,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>382</v>
+      </c>
+      <c r="B18" t="s">
         <v>383</v>
-      </c>
-      <c r="B18" t="s">
-        <v>384</v>
       </c>
       <c r="C18">
         <v>120</v>
@@ -6348,12 +6345,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B19" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C19">
         <v>30</v>
@@ -6362,12 +6359,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B20" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C20">
         <v>90</v>
@@ -6382,25 +6379,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9a4568ba-f362-4e84-99d7-dc60d25416b3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E9B12C2B262A7D41BAA1C1A05186961E" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c5712268625b41a295c1c13b9cc08810">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9a4568ba-f362-4e84-99d7-dc60d25416b3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2284d5a418b13d67f420d8f33de3453b" ns2:_="">
     <xsd:import namespace="9a4568ba-f362-4e84-99d7-dc60d25416b3"/>
@@ -6572,14 +6550,57 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9a4568ba-f362-4e84-99d7-dc60d25416b3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58E57473-BAD3-4CDA-A67F-19CDC21767EF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D5C309B-A406-4F09-B9ED-A6A4D616E23D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9a4568ba-f362-4e84-99d7-dc60d25416b3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8ED54FA-4DB1-4C56-A86D-28FB7FDDBA5D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8ED54FA-4DB1-4C56-A86D-28FB7FDDBA5D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D5C309B-A406-4F09-B9ED-A6A4D616E23D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58E57473-BAD3-4CDA-A67F-19CDC21767EF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9a4568ba-f362-4e84-99d7-dc60d25416b3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>